<commit_message>
Flash v5.65: Weekly Flash Sales + Live Ent through Week 38
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/live-entertainment-report-2026.xlsx
+++ b/data/excel/live-entertainment-report-2026.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56339578-2CD3-4D61-B4BA-67C524CB7F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C20D5429-ABA9-42F7-9E75-A32CE52124C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4 - Casa Neos" sheetId="1" r:id="rId1"/>
     <sheet name="11 - CN Lounge Rooftop" sheetId="2" r:id="rId2"/>
-    <sheet name="10 - Mila II MM Club" sheetId="3" r:id="rId3"/>
+    <sheet name="10 - Mila II MM Club" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'10 - Mila II MM Club'!#REF!</definedName>
@@ -54,7 +54,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>09/08/2026 10:41 AM PDT</t>
+    <t>09/21/2026 06:38 AM PDT</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -455,9 +455,15 @@
     <col min="16" max="16" width="1.42578125" customWidth="1"/>
     <col min="17" max="17" width="17.140625" customWidth="1"/>
     <col min="18" max="18" width="9.42578125" customWidth="1"/>
+    <col min="19" max="19" width="1.42578125" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" customWidth="1"/>
+    <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -502,8 +508,22 @@
       <c r="R1" s="7">
         <v>0.99999999999999989</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S1" s="1"/>
+      <c r="T1" s="6">
+        <v>417790.01</v>
+      </c>
+      <c r="U1" s="7">
+        <v>1</v>
+      </c>
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>406693.96</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -536,20 +556,34 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>26167.13</v>
+        <v>27517.13</v>
       </c>
       <c r="O2" s="4">
-        <v>6.3855828424167899E-2</v>
+        <v>6.715024276661305E-2</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>7662.95</v>
+        <v>13173.34</v>
       </c>
       <c r="R2" s="4">
-        <v>2.0182967976561158E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>3.4696441887830692E-2</v>
+      </c>
+      <c r="S2" s="5"/>
+      <c r="T2" s="3">
+        <v>28096.59</v>
+      </c>
+      <c r="U2" s="4">
+        <v>6.7250507019064432E-2</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>16503.25</v>
+      </c>
+      <c r="X2" s="4">
+        <v>4.0579038842868481E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -582,18 +616,28 @@
         <v>379674.09</v>
       </c>
       <c r="R3" s="10"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S3" s="5"/>
+      <c r="T3" s="3">
+        <v>417790.01</v>
+      </c>
+      <c r="U3" s="10"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>406693.96</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -608,7 +652,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -629,9 +673,15 @@
     <col min="16" max="16" width="1.42578125" customWidth="1"/>
     <col min="17" max="17" width="17.140625" customWidth="1"/>
     <col min="18" max="18" width="9.42578125" customWidth="1"/>
+    <col min="19" max="19" width="1.42578125" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" customWidth="1"/>
+    <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -676,8 +726,22 @@
       <c r="R1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S1" s="1"/>
+      <c r="T1" s="6">
+        <v>108804</v>
+      </c>
+      <c r="U1" s="7">
+        <v>1</v>
+      </c>
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>35776</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -710,20 +774,34 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>-2150</v>
+        <v>7814.25</v>
       </c>
       <c r="O2" s="4">
-        <v>-2.3150179521566543E-2</v>
+        <v>8.4140135035535524E-2</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>1300</v>
+        <v>6519.12</v>
       </c>
       <c r="R2" s="4">
-        <v>8.4755763228907717E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>4.2502537783141295E-2</v>
+      </c>
+      <c r="S2" s="5"/>
+      <c r="T2" s="3">
+        <v>5100</v>
+      </c>
+      <c r="U2" s="4">
+        <v>4.6873276717767733E-2</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>0</v>
+      </c>
+      <c r="X2" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -756,18 +834,28 @@
         <v>153381.9</v>
       </c>
       <c r="R3" s="10"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S3" s="5"/>
+      <c r="T3" s="3">
+        <v>108804</v>
+      </c>
+      <c r="U3" s="10"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>35776</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -778,11 +866,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -803,9 +891,15 @@
     <col min="16" max="16" width="1.42578125" customWidth="1"/>
     <col min="17" max="17" width="17.140625" customWidth="1"/>
     <col min="18" max="18" width="9.42578125" customWidth="1"/>
+    <col min="19" max="19" width="1.42578125" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" customWidth="1"/>
+    <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -845,13 +939,27 @@
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="6">
-        <v>289553.25</v>
+        <v>290229.07</v>
       </c>
       <c r="R1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S1" s="1"/>
+      <c r="T1" s="6">
+        <v>161195.03</v>
+      </c>
+      <c r="U1" s="7">
+        <v>1</v>
+      </c>
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>276926</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -884,20 +992,34 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>11290</v>
+        <v>15990</v>
       </c>
       <c r="O2" s="4">
-        <v>4.8271274816149075E-2</v>
+        <v>6.8366491081507857E-2</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>14400</v>
+        <v>20700</v>
       </c>
       <c r="R2" s="4">
-        <v>4.9731785086162911E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>7.1322972574732094E-2</v>
+      </c>
+      <c r="S2" s="5"/>
+      <c r="T2" s="3">
+        <v>17440.04</v>
+      </c>
+      <c r="U2" s="4">
+        <v>0.10819216944840049</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>7900</v>
+      </c>
+      <c r="X2" s="4">
+        <v>2.8527476654413093E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -927,21 +1049,31 @@
       <c r="O3" s="10"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="3">
-        <v>289553.25</v>
+        <v>290229.07</v>
       </c>
       <c r="R3" s="10"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S3" s="5"/>
+      <c r="T3" s="3">
+        <v>161195.03</v>
+      </c>
+      <c r="U3" s="10"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>276926</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Flash v5.69: Weekly Flash Sales + Live Ent through Week 39
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/live-entertainment-report-2026.xlsx
+++ b/data/excel/live-entertainment-report-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C20D5429-ABA9-42F7-9E75-A32CE52124C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{58459C0A-5521-4BCB-8A53-9DF4BCA76591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4 - Casa Neos" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>09/21/2026 06:38 AM PDT</t>
+    <t>09/28/2026 01:57 PM PDT</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -461,9 +461,12 @@
     <col min="22" max="22" width="1.42578125" customWidth="1"/>
     <col min="23" max="23" width="17.140625" customWidth="1"/>
     <col min="24" max="24" width="9.42578125" customWidth="1"/>
+    <col min="25" max="25" width="1.42578125" customWidth="1"/>
+    <col min="26" max="26" width="17.140625" customWidth="1"/>
+    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -503,14 +506,14 @@
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="6">
-        <v>379674.08999999997</v>
+        <v>376870.35</v>
       </c>
       <c r="R1" s="7">
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
       <c r="S1" s="1"/>
       <c r="T1" s="6">
-        <v>417790.01</v>
+        <v>415663.37</v>
       </c>
       <c r="U1" s="7">
         <v>1</v>
@@ -522,8 +525,15 @@
       <c r="X1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="6">
+        <v>457563.8</v>
+      </c>
+      <c r="AA1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -566,24 +576,31 @@
         <v>13173.34</v>
       </c>
       <c r="R2" s="4">
-        <v>3.4696441887830692E-2</v>
+        <v>3.4954567266965948E-2</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
-        <v>28096.59</v>
+        <v>31271.59</v>
       </c>
       <c r="U2" s="4">
-        <v>6.7250507019064432E-2</v>
+        <v>7.5232970372154762E-2</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="3">
-        <v>16503.25</v>
+        <v>21364.13</v>
       </c>
       <c r="X2" s="4">
-        <v>4.0579038842868481E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>5.2531220281707654E-2</v>
+      </c>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="3">
+        <v>7830.03</v>
+      </c>
+      <c r="AA2" s="4">
+        <v>1.7112433282528032E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -613,12 +630,12 @@
       <c r="O3" s="10"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="3">
-        <v>379674.09</v>
+        <v>376870.35</v>
       </c>
       <c r="R3" s="10"/>
       <c r="S3" s="5"/>
       <c r="T3" s="3">
-        <v>417790.01</v>
+        <v>415663.37</v>
       </c>
       <c r="U3" s="10"/>
       <c r="V3" s="5"/>
@@ -626,18 +643,23 @@
         <v>406693.96</v>
       </c>
       <c r="X3" s="10"/>
-    </row>
-    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="3">
+        <v>457563.8</v>
+      </c>
+      <c r="AA3" s="10"/>
+    </row>
+    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -652,7 +674,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -679,9 +701,12 @@
     <col min="22" max="22" width="1.42578125" customWidth="1"/>
     <col min="23" max="23" width="17.140625" customWidth="1"/>
     <col min="24" max="24" width="9.42578125" customWidth="1"/>
+    <col min="25" max="25" width="1.42578125" customWidth="1"/>
+    <col min="26" max="26" width="17.140625" customWidth="1"/>
+    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -721,7 +746,7 @@
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="6">
-        <v>153381.9</v>
+        <v>153190.5</v>
       </c>
       <c r="R1" s="7">
         <v>1</v>
@@ -740,8 +765,15 @@
       <c r="X1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="6">
+        <v>131170.23000000001</v>
+      </c>
+      <c r="AA1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -784,24 +816,31 @@
         <v>6519.12</v>
       </c>
       <c r="R2" s="4">
-        <v>4.2502537783141295E-2</v>
+        <v>4.2555641505184719E-2</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
-        <v>5100</v>
+        <v>5775</v>
       </c>
       <c r="U2" s="4">
-        <v>4.6873276717767733E-2</v>
+        <v>5.3077092753942873E-2</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="3">
+        <v>600</v>
+      </c>
+      <c r="X2" s="4">
+        <v>1.6771019677996421E-2</v>
+      </c>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="3">
         <v>0</v>
       </c>
-      <c r="X2" s="4">
+      <c r="AA2" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -831,7 +870,7 @@
       <c r="O3" s="10"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="3">
-        <v>153381.9</v>
+        <v>153190.5</v>
       </c>
       <c r="R3" s="10"/>
       <c r="S3" s="5"/>
@@ -844,18 +883,23 @@
         <v>35776</v>
       </c>
       <c r="X3" s="10"/>
-    </row>
-    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="3">
+        <v>131170.23000000001</v>
+      </c>
+      <c r="AA3" s="10"/>
+    </row>
+    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -870,7 +914,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -897,9 +941,12 @@
     <col min="22" max="22" width="1.42578125" customWidth="1"/>
     <col min="23" max="23" width="17.140625" customWidth="1"/>
     <col min="24" max="24" width="9.42578125" customWidth="1"/>
+    <col min="25" max="25" width="1.42578125" customWidth="1"/>
+    <col min="26" max="26" width="17.140625" customWidth="1"/>
+    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -953,13 +1000,20 @@
       </c>
       <c r="V1" s="1"/>
       <c r="W1" s="6">
-        <v>276926</v>
+        <v>278686</v>
       </c>
       <c r="X1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="6">
+        <v>267581.59999999998</v>
+      </c>
+      <c r="AA1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -992,17 +1046,17 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>15990</v>
+        <v>18390</v>
       </c>
       <c r="O2" s="4">
-        <v>6.8366491081507857E-2</v>
+        <v>7.8627878110627242E-2</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>20700</v>
+        <v>21000</v>
       </c>
       <c r="R2" s="4">
-        <v>7.1322972574732094E-2</v>
+        <v>7.2356638843931106E-2</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
@@ -1013,13 +1067,20 @@
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="3">
-        <v>7900</v>
+        <v>17678.25</v>
       </c>
       <c r="X2" s="4">
-        <v>2.8527476654413093E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>6.3434295228321474E-2</v>
+      </c>
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="3">
+        <v>3000</v>
+      </c>
+      <c r="AA2" s="4">
+        <v>1.1211533229489623E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -1059,21 +1120,26 @@
       <c r="U3" s="10"/>
       <c r="V3" s="5"/>
       <c r="W3" s="3">
-        <v>276926</v>
+        <v>278686</v>
       </c>
       <c r="X3" s="10"/>
-    </row>
-    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="3">
+        <v>267581.59999999998</v>
+      </c>
+      <c r="AA3" s="10"/>
+    </row>
+    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Flash v5.74: Weekly Flash Sales + Live Ent through Week 40
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/live-entertainment-report-2026.xlsx
+++ b/data/excel/live-entertainment-report-2026.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58459C0A-5521-4BCB-8A53-9DF4BCA76591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B929702-57F0-419B-8555-352C8B2E6D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="855" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4 - Casa Neos" sheetId="1" r:id="rId1"/>
     <sheet name="11 - CN Lounge Rooftop" sheetId="2" r:id="rId2"/>
-    <sheet name="10 - Mila II MM Club" sheetId="4" r:id="rId3"/>
+    <sheet name="10 - Mila II MM Club" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'10 - Mila II MM Club'!#REF!</definedName>
@@ -54,7 +54,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>09/28/2026 01:57 PM PDT</t>
+    <t>10/05/2026 06:57 AM PDT</t>
   </si>
 </sst>
 </file>
@@ -76,12 +76,14 @@
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -89,12 +91,14 @@
       <i/>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -434,7 +438,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -452,220 +456,150 @@
     <col min="13" max="13" width="1.42578125" customWidth="1"/>
     <col min="14" max="14" width="17.140625" customWidth="1"/>
     <col min="15" max="15" width="9.42578125" customWidth="1"/>
-    <col min="16" max="16" width="1.42578125" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" customWidth="1"/>
-    <col min="18" max="18" width="9.42578125" customWidth="1"/>
-    <col min="19" max="19" width="1.42578125" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" customWidth="1"/>
-    <col min="21" max="21" width="9.42578125" customWidth="1"/>
-    <col min="22" max="22" width="1.42578125" customWidth="1"/>
-    <col min="23" max="23" width="17.140625" customWidth="1"/>
-    <col min="24" max="24" width="9.42578125" customWidth="1"/>
-    <col min="25" max="25" width="1.42578125" customWidth="1"/>
-    <col min="26" max="26" width="17.140625" customWidth="1"/>
-    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6">
-        <v>319662.52</v>
-      </c>
-      <c r="C1" s="7">
-        <v>1</v>
+      <c r="B1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="C1" s="7" t="str">
+        <f>IFERROR(B1/B3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="D1" s="1"/>
-      <c r="E1" s="6">
-        <v>439726.29000000004</v>
-      </c>
-      <c r="F1" s="7">
-        <v>1.0000000000000002</v>
+      <c r="E1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="F1" s="7" t="str">
+        <f>IFERROR(E1/E3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="G1" s="1"/>
-      <c r="H1" s="6">
-        <v>372907.44</v>
-      </c>
-      <c r="I1" s="7">
-        <v>1</v>
+      <c r="H1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="I1" s="7" t="str">
+        <f>IFERROR(H1/H3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="J1" s="1"/>
-      <c r="K1" s="6">
-        <v>381892.96</v>
-      </c>
-      <c r="L1" s="7">
-        <v>1</v>
+      <c r="K1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="L1" s="7" t="str">
+        <f>IFERROR(K1/K3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="M1" s="1"/>
-      <c r="N1" s="6">
-        <v>409784.51999999996</v>
-      </c>
-      <c r="O1" s="7">
-        <v>0.99999999999999989</v>
-      </c>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="6">
-        <v>376870.35</v>
-      </c>
-      <c r="R1" s="7">
-        <v>1</v>
-      </c>
-      <c r="S1" s="1"/>
-      <c r="T1" s="6">
-        <v>415663.37</v>
-      </c>
-      <c r="U1" s="7">
-        <v>1</v>
-      </c>
-      <c r="V1" s="1"/>
-      <c r="W1" s="6">
-        <v>406693.96</v>
-      </c>
-      <c r="X1" s="7">
-        <v>1</v>
-      </c>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="6">
-        <v>457563.8</v>
-      </c>
-      <c r="AA1" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="O1" s="7" t="str">
+        <f>IFERROR(N1/N3, "NA")</f>
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>14158.87</v>
+        <v>11373.34</v>
       </c>
       <c r="C2" s="4">
-        <v>4.4293181446482997E-2</v>
+        <f>IFERROR(B2/B3, "NA")</f>
+        <v>3.0178388934019355E-2</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="3">
-        <v>28883.95</v>
+        <v>32365.34</v>
       </c>
       <c r="F2" s="4">
-        <v>6.5686202205467406E-2</v>
+        <f>IFERROR(E2/E3, "NA")</f>
+        <v>7.7864306397746816E-2</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3">
-        <v>18686.55</v>
+        <v>22364.13</v>
       </c>
       <c r="I2" s="4">
-        <v>5.0110424184618037E-2</v>
+        <f>IFERROR(H2/H3, "NA")</f>
+        <v>5.4990071649945328E-2</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="3">
-        <v>25748.31</v>
+        <v>10395.56</v>
       </c>
       <c r="L2" s="4">
-        <v>6.7422845396259729E-2</v>
+        <f>IFERROR(K2/K3, "NA")</f>
+        <v>2.2719367222669276E-2</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>27517.13</v>
+        <v>13700</v>
       </c>
       <c r="O2" s="4">
-        <v>6.715024276661305E-2</v>
-      </c>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="3">
-        <v>13173.34</v>
-      </c>
-      <c r="R2" s="4">
-        <v>3.4954567266965948E-2</v>
-      </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="3">
-        <v>31271.59</v>
-      </c>
-      <c r="U2" s="4">
-        <v>7.5232970372154762E-2</v>
-      </c>
-      <c r="V2" s="5"/>
-      <c r="W2" s="3">
-        <v>21364.13</v>
-      </c>
-      <c r="X2" s="4">
-        <v>5.2531220281707654E-2</v>
-      </c>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="3">
-        <v>7830.03</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>1.7112433282528032E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <f>IFERROR(N2/N3, "NA")</f>
+        <v>3.0014498098000972E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3">
-        <v>319662.52</v>
+        <v>376870.35</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="5"/>
       <c r="E3" s="3">
-        <v>439726.29</v>
+        <v>415663.37</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="5"/>
       <c r="H3" s="3">
-        <v>372907.44</v>
+        <v>406693.96</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="5"/>
       <c r="K3" s="3">
-        <v>381892.96</v>
+        <v>457563.8</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="5"/>
       <c r="N3" s="3">
-        <v>409784.52</v>
+        <v>456446.08</v>
       </c>
       <c r="O3" s="10"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="3">
-        <v>376870.35</v>
-      </c>
-      <c r="R3" s="10"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="3">
-        <v>415663.37</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="3">
-        <v>406693.96</v>
-      </c>
-      <c r="X3" s="10"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="3">
-        <v>457563.8</v>
-      </c>
-      <c r="AA3" s="10"/>
-    </row>
-    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:O1 A3:O8 A2:O2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -674,7 +608,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -692,229 +626,159 @@
     <col min="13" max="13" width="1.42578125" customWidth="1"/>
     <col min="14" max="14" width="17.140625" customWidth="1"/>
     <col min="15" max="15" width="9.42578125" customWidth="1"/>
-    <col min="16" max="16" width="1.42578125" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" customWidth="1"/>
-    <col min="18" max="18" width="9.42578125" customWidth="1"/>
-    <col min="19" max="19" width="1.42578125" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" customWidth="1"/>
-    <col min="21" max="21" width="9.42578125" customWidth="1"/>
-    <col min="22" max="22" width="1.42578125" customWidth="1"/>
-    <col min="23" max="23" width="17.140625" customWidth="1"/>
-    <col min="24" max="24" width="9.42578125" customWidth="1"/>
-    <col min="25" max="25" width="1.42578125" customWidth="1"/>
-    <col min="26" max="26" width="17.140625" customWidth="1"/>
-    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6">
-        <v>49573</v>
-      </c>
-      <c r="C1" s="7">
-        <v>1</v>
+      <c r="B1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="C1" s="7" t="str">
+        <f>IFERROR(B1/B3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="D1" s="1"/>
-      <c r="E1" s="6">
-        <v>84397</v>
-      </c>
-      <c r="F1" s="7">
-        <v>1</v>
+      <c r="E1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="F1" s="7" t="str">
+        <f>IFERROR(E1/E3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="G1" s="1"/>
-      <c r="H1" s="6">
-        <v>145999.85999999999</v>
-      </c>
-      <c r="I1" s="7">
-        <v>1</v>
+      <c r="H1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="I1" s="7" t="str">
+        <f>IFERROR(H1/H3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="J1" s="1"/>
-      <c r="K1" s="6">
-        <v>175395.55</v>
-      </c>
-      <c r="L1" s="7">
-        <v>1</v>
+      <c r="K1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="L1" s="7" t="str">
+        <f>IFERROR(K1/K3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="M1" s="1"/>
-      <c r="N1" s="6">
-        <v>92871.85</v>
-      </c>
-      <c r="O1" s="7">
-        <v>1</v>
-      </c>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="6">
-        <v>153190.5</v>
-      </c>
-      <c r="R1" s="7">
-        <v>1</v>
-      </c>
-      <c r="S1" s="1"/>
-      <c r="T1" s="6">
-        <v>108804</v>
-      </c>
-      <c r="U1" s="7">
-        <v>1</v>
-      </c>
-      <c r="V1" s="1"/>
-      <c r="W1" s="6">
-        <v>35776</v>
-      </c>
-      <c r="X1" s="7">
-        <v>1</v>
-      </c>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="6">
-        <v>131170.23000000001</v>
-      </c>
-      <c r="AA1" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="O1" s="7" t="str">
+        <f>IFERROR(N1/N3, "NA")</f>
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>2650</v>
+        <v>6519.12</v>
       </c>
       <c r="C2" s="4">
-        <v>5.3456518669436993E-2</v>
+        <f>IFERROR(B2/B3, "NA")</f>
+        <v>4.2555641505184719E-2</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="3">
-        <v>9876.81</v>
+        <v>22015</v>
       </c>
       <c r="F2" s="4">
-        <v>0.11702797492801877</v>
+        <f>IFERROR(E2/E3, "NA")</f>
+        <v>0.2023363111650307</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3">
-        <v>9750</v>
+        <v>600</v>
       </c>
       <c r="I2" s="4">
-        <v>6.6780885954274213E-2</v>
+        <f>IFERROR(H2/H3, "NA")</f>
+        <v>1.6771019677996421E-2</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="3">
-        <v>9739.36</v>
+        <v>5400</v>
       </c>
       <c r="L2" s="4">
-        <v>5.552797662198386E-2</v>
+        <f>IFERROR(K2/K3, "NA")</f>
+        <v>4.1167877802760579E-2</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>7814.25</v>
+        <v>25100</v>
       </c>
       <c r="O2" s="4">
-        <v>8.4140135035535524E-2</v>
-      </c>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="3">
-        <v>6519.12</v>
-      </c>
-      <c r="R2" s="4">
-        <v>4.2555641505184719E-2</v>
-      </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="3">
-        <v>5775</v>
-      </c>
-      <c r="U2" s="4">
-        <v>5.3077092753942873E-2</v>
-      </c>
-      <c r="V2" s="5"/>
-      <c r="W2" s="3">
-        <v>600</v>
-      </c>
-      <c r="X2" s="4">
-        <v>1.6771019677996421E-2</v>
-      </c>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <f>IFERROR(N2/N3, "NA")</f>
+        <v>0.18988718356076295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3">
-        <v>49573</v>
+        <v>153190.5</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="5"/>
       <c r="E3" s="3">
-        <v>84397</v>
+        <v>108804</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="5"/>
       <c r="H3" s="3">
-        <v>145999.85999999999</v>
+        <v>35776</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="5"/>
       <c r="K3" s="3">
-        <v>175395.55</v>
+        <v>131170.23000000001</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="5"/>
       <c r="N3" s="3">
-        <v>92871.85</v>
+        <v>132183.75</v>
       </c>
       <c r="O3" s="10"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="3">
-        <v>153190.5</v>
-      </c>
-      <c r="R3" s="10"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="3">
-        <v>108804</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="3">
-        <v>35776</v>
-      </c>
-      <c r="X3" s="10"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="3">
-        <v>131170.23000000001</v>
-      </c>
-      <c r="AA3" s="10"/>
-    </row>
-    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:O1 A3:O8 A2:O2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -932,219 +796,149 @@
     <col min="13" max="13" width="1.42578125" customWidth="1"/>
     <col min="14" max="14" width="17.140625" customWidth="1"/>
     <col min="15" max="15" width="9.42578125" customWidth="1"/>
-    <col min="16" max="16" width="1.42578125" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" customWidth="1"/>
-    <col min="18" max="18" width="9.42578125" customWidth="1"/>
-    <col min="19" max="19" width="1.42578125" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" customWidth="1"/>
-    <col min="21" max="21" width="9.42578125" customWidth="1"/>
-    <col min="22" max="22" width="1.42578125" customWidth="1"/>
-    <col min="23" max="23" width="17.140625" customWidth="1"/>
-    <col min="24" max="24" width="9.42578125" customWidth="1"/>
-    <col min="25" max="25" width="1.42578125" customWidth="1"/>
-    <col min="26" max="26" width="17.140625" customWidth="1"/>
-    <col min="27" max="27" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6">
-        <v>66507</v>
-      </c>
-      <c r="C1" s="7">
-        <v>1</v>
+      <c r="B1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="C1" s="7" t="str">
+        <f>IFERROR(B1/B3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="D1" s="1"/>
-      <c r="E1" s="6">
-        <v>176817.5</v>
-      </c>
-      <c r="F1" s="7">
-        <v>1</v>
+      <c r="E1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="F1" s="7" t="str">
+        <f>IFERROR(E1/E3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="G1" s="1"/>
-      <c r="H1" s="6">
-        <v>168912</v>
-      </c>
-      <c r="I1" s="7">
-        <v>1</v>
+      <c r="H1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="I1" s="7" t="str">
+        <f>IFERROR(H1/H3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="J1" s="1"/>
-      <c r="K1" s="6">
-        <v>302980.79000000004</v>
-      </c>
-      <c r="L1" s="7">
-        <v>1.0000000000000002</v>
+      <c r="K1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="L1" s="7" t="str">
+        <f>IFERROR(K1/K3, "NA")</f>
+        <v>NA</v>
       </c>
       <c r="M1" s="1"/>
-      <c r="N1" s="6">
-        <v>233886.51</v>
-      </c>
-      <c r="O1" s="7">
-        <v>1</v>
-      </c>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="6">
-        <v>290229.07</v>
-      </c>
-      <c r="R1" s="7">
-        <v>1</v>
-      </c>
-      <c r="S1" s="1"/>
-      <c r="T1" s="6">
-        <v>161195.03</v>
-      </c>
-      <c r="U1" s="7">
-        <v>1</v>
-      </c>
-      <c r="V1" s="1"/>
-      <c r="W1" s="6">
-        <v>278686</v>
-      </c>
-      <c r="X1" s="7">
-        <v>1</v>
-      </c>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="6">
-        <v>267581.59999999998</v>
-      </c>
-      <c r="AA1" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="6" t="str">
+        <f>IFERROR(#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!+#REF!, "NA")</f>
+        <v>NA</v>
+      </c>
+      <c r="O1" s="7" t="str">
+        <f>IFERROR(N1/N3, "NA")</f>
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>3300</v>
+        <v>25000</v>
       </c>
       <c r="C2" s="4">
-        <v>4.9618837114890159E-2</v>
+        <f>IFERROR(B2/B3, "NA")</f>
+        <v>8.6138855766584643E-2</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="3">
-        <v>20035</v>
+        <v>19440.04</v>
       </c>
       <c r="F2" s="4">
-        <v>0.1133089202143453</v>
+        <f>IFERROR(E2/E3, "NA")</f>
+        <v>0.12059949987291793</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3">
-        <v>19300</v>
+        <v>17678.25</v>
       </c>
       <c r="I2" s="4">
-        <v>0.11426068011745762</v>
+        <f>IFERROR(H2/H3, "NA")</f>
+        <v>6.3434295228321474E-2</v>
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="3">
-        <v>32932.44</v>
+        <v>13299.18</v>
       </c>
       <c r="L2" s="4">
-        <v>0.10869481197141247</v>
+        <f>IFERROR(K2/K3, "NA")</f>
+        <v>4.9701399498321266E-2</v>
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>18390</v>
+        <v>8100</v>
       </c>
       <c r="O2" s="4">
-        <v>7.8627878110627242E-2</v>
-      </c>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="3">
-        <v>21000</v>
-      </c>
-      <c r="R2" s="4">
-        <v>7.2356638843931106E-2</v>
-      </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="3">
-        <v>17440.04</v>
-      </c>
-      <c r="U2" s="4">
-        <v>0.10819216944840049</v>
-      </c>
-      <c r="V2" s="5"/>
-      <c r="W2" s="3">
-        <v>17678.25</v>
-      </c>
-      <c r="X2" s="4">
-        <v>6.3434295228321474E-2</v>
-      </c>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="3">
-        <v>3000</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>1.1211533229489623E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <f>IFERROR(N2/N3, "NA")</f>
+        <v>2.4190493506375598E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3">
-        <v>66507</v>
+        <v>290229.07</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="5"/>
       <c r="E3" s="3">
-        <v>176817.5</v>
+        <v>161195.03</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="5"/>
       <c r="H3" s="3">
-        <v>168912</v>
+        <v>278686</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="5"/>
       <c r="K3" s="3">
-        <v>302980.78999999998</v>
+        <v>267581.59999999998</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="5"/>
       <c r="N3" s="3">
-        <v>233886.51</v>
+        <v>334842.28000000003</v>
       </c>
       <c r="O3" s="10"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="3">
-        <v>290229.07</v>
-      </c>
-      <c r="R3" s="10"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="3">
-        <v>161195.03</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="3">
-        <v>278686</v>
-      </c>
-      <c r="X3" s="10"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="3">
-        <v>267581.59999999998</v>
-      </c>
-      <c r="AA3" s="10"/>
-    </row>
-    <row r="6" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:O1 A3:O8 A2:O2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flash v5.112: update sales and live entertainment through week 43
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/excel/live-entertainment-report-2026.xlsx
+++ b/data/excel/live-entertainment-report-2026.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatthiasLavenant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30F57DCE-DE9B-459A-85E8-A7F17C3132A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{36B05A43-6A8D-4CF1-B134-5864E8A07DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4 - Casa Neos" sheetId="1" r:id="rId1"/>
     <sheet name="11 - CN Lounge Rooftop" sheetId="2" r:id="rId2"/>
-    <sheet name="10 - Mila II MM Club" sheetId="3" r:id="rId3"/>
+    <sheet name="10 - Mila II MM Club" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'10 - Mila II MM Club'!#REF!</definedName>
@@ -54,7 +54,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>10/19/2026 01:55 PM PDT</t>
+    <t>10/26/2026 06:43 AM PDT</t>
   </si>
 </sst>
 </file>
@@ -76,14 +76,12 @@
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -91,14 +89,12 @@
       <i/>
       <sz val="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -438,7 +434,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -462,9 +458,12 @@
     <col min="19" max="19" width="1.42578125" customWidth="1"/>
     <col min="20" max="20" width="17.140625" customWidth="1"/>
     <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -516,8 +515,15 @@
       <c r="U1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>504154.99</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -557,20 +563,27 @@
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>76714.289999999994</v>
+        <v>77164.289999999994</v>
       </c>
       <c r="R2" s="4">
-        <v>0.12823619696279245</v>
+        <v>0.12898842042250586</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
-        <v>46550</v>
+        <v>48908.73</v>
       </c>
       <c r="U2" s="4">
-        <v>7.5876489180012635E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>7.9721218531754234E-2</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>27500</v>
+      </c>
+      <c r="X2" s="4">
+        <v>5.4546717865472286E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -608,18 +621,23 @@
         <v>613497.02</v>
       </c>
       <c r="U3" s="10"/>
-    </row>
-    <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>504154.99</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -634,7 +652,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -658,9 +676,12 @@
     <col min="19" max="19" width="1.42578125" customWidth="1"/>
     <col min="20" max="20" width="17.140625" customWidth="1"/>
     <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -712,8 +733,15 @@
       <c r="U1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>146420.31</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -746,10 +774,10 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="3">
-        <v>29950</v>
+        <v>30350</v>
       </c>
       <c r="O2" s="4">
-        <v>0.22657853177867929</v>
+        <v>0.22960462235335283</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
@@ -760,13 +788,20 @@
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
-        <v>7798.89</v>
+        <v>38798.89</v>
       </c>
       <c r="U2" s="4">
-        <v>4.3520287944420033E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.21651015269145724</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>24100</v>
+      </c>
+      <c r="X2" s="4">
+        <v>0.1645946522036458</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -804,18 +839,23 @@
         <v>179201.25</v>
       </c>
       <c r="U3" s="10"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>146420.31</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
@@ -826,11 +866,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
@@ -854,9 +894,12 @@
     <col min="19" max="19" width="1.42578125" customWidth="1"/>
     <col min="20" max="20" width="17.140625" customWidth="1"/>
     <col min="21" max="21" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="1.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.140625" customWidth="1"/>
+    <col min="24" max="24" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -903,13 +946,20 @@
       </c>
       <c r="S1" s="1"/>
       <c r="T1" s="6">
-        <v>293067.86</v>
+        <v>292755.86</v>
       </c>
       <c r="U1" s="7">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V1" s="1"/>
+      <c r="W1" s="6">
+        <v>423090.8</v>
+      </c>
+      <c r="X1" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -949,20 +999,27 @@
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="3">
-        <v>60723.96</v>
+        <v>69023.960000000006</v>
       </c>
       <c r="R2" s="4">
-        <v>0.18385010048726788</v>
+        <v>0.20897948654911769</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="3">
-        <v>34775</v>
+        <v>40214.800000000003</v>
       </c>
       <c r="U2" s="4">
-        <v>0.11865852502556917</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.13736633657819866</v>
+      </c>
+      <c r="V2" s="5"/>
+      <c r="W2" s="3">
+        <v>12634.83</v>
+      </c>
+      <c r="X2" s="4">
+        <v>2.9863164124580351E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
@@ -997,21 +1054,26 @@
       <c r="R3" s="10"/>
       <c r="S3" s="5"/>
       <c r="T3" s="3">
-        <v>293067.86</v>
+        <v>292755.86</v>
       </c>
       <c r="U3" s="10"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V3" s="5"/>
+      <c r="W3" s="3">
+        <v>423090.8</v>
+      </c>
+      <c r="X3" s="10"/>
+    </row>
+    <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>4</v>
       </c>

</xml_diff>